<commit_message>
datos con 3 cifras significativas
</commit_message>
<xml_diff>
--- a/Datos ESPARTACO/Parámetros para análisis de Antares/resultados perfiles halpha 2025 y 2026.xlsx
+++ b/Datos ESPARTACO/Parámetros para análisis de Antares/resultados perfiles halpha 2025 y 2026.xlsx
@@ -482,7 +482,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6562.2305</v>
+        <v>6562.231</v>
       </c>
       <c r="D2" t="n">
         <v>-8.899999999999999e-05</v>
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>6563.0012</v>
+        <v>6563.001</v>
       </c>
       <c r="D3" t="n">
         <v>2.9e-05</v>
@@ -542,7 +542,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>6562.4528</v>
+        <v>6562.453</v>
       </c>
       <c r="D4" t="n">
         <v>-5.5e-05</v>
@@ -572,7 +572,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6563.0682</v>
+        <v>6563.068</v>
       </c>
       <c r="D5" t="n">
         <v>3.9e-05</v>
@@ -602,7 +602,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6562.4692</v>
+        <v>6562.469</v>
       </c>
       <c r="D6" t="n">
         <v>-5.2e-05</v>
@@ -632,7 +632,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>6562.9478</v>
+        <v>6562.948</v>
       </c>
       <c r="D7" t="n">
         <v>2.1e-05</v>

</xml_diff>

<commit_message>
Adición a la tabla de excel los parámetros de la línea de Cobalto c:
</commit_message>
<xml_diff>
--- a/Datos ESPARTACO/Parámetros para análisis de Antares/resultados perfiles halpha 2025 y 2026.xlsx
+++ b/Datos ESPARTACO/Parámetros para análisis de Antares/resultados perfiles halpha 2025 y 2026.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -533,31 +533,31 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Agosto-2026</t>
+          <t>Julio-2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Emisión Azul Hα</t>
+          <t>Absorción Cobalto</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>6562.453</v>
+        <v>6563.901</v>
       </c>
       <c r="D4" t="n">
-        <v>-5.5e-05</v>
+        <v>7.7e-05</v>
       </c>
       <c r="E4" t="n">
-        <v>-16.4071</v>
+        <v>23</v>
       </c>
       <c r="F4" t="n">
-        <v>0.6014</v>
+        <v>0.3432</v>
       </c>
       <c r="G4" t="n">
-        <v>1.273</v>
+        <v>0.925</v>
       </c>
       <c r="H4" t="n">
-        <v>0.9461000000000001</v>
+        <v>0.4043</v>
       </c>
     </row>
     <row r="5">
@@ -568,86 +568,176 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Absorción Hα</t>
+          <t>Emisión Azul Hα</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6563.068</v>
+        <v>6562.453</v>
       </c>
       <c r="D5" t="n">
-        <v>3.9e-05</v>
+        <v>-5.5e-05</v>
       </c>
       <c r="E5" t="n">
-        <v>11.7029</v>
+        <v>-16.4071</v>
       </c>
       <c r="F5" t="n">
-        <v>1.033</v>
+        <v>0.6014</v>
       </c>
       <c r="G5" t="n">
-        <v>1.375</v>
+        <v>1.273</v>
       </c>
       <c r="H5" t="n">
-        <v>1.8256</v>
+        <v>0.9461000000000001</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Septiembre-2025</t>
+          <t>Agosto-2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Emisión Azul Hα</t>
+          <t>Absorción Hα</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6562.469</v>
+        <v>6563.068</v>
       </c>
       <c r="D6" t="n">
-        <v>-5.2e-05</v>
+        <v>3.9e-05</v>
       </c>
       <c r="E6" t="n">
-        <v>-15.6611</v>
+        <v>11.7029</v>
       </c>
       <c r="F6" t="n">
-        <v>0.8374</v>
+        <v>1.033</v>
       </c>
       <c r="G6" t="n">
-        <v>1.313</v>
+        <v>1.375</v>
       </c>
       <c r="H6" t="n">
-        <v>1.4598</v>
+        <v>1.8256</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Agosto-2026</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>6564.025</v>
+      </c>
+      <c r="D7" t="n">
+        <v>9.6e-05</v>
+      </c>
+      <c r="E7" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.4175</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.3948</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>Septiembre-2025</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Emisión Azul Hα</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>6562.469</v>
+      </c>
+      <c r="D8" t="n">
+        <v>-5.2e-05</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-15.6611</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.8374</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1.313</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1.4598</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Septiembre-2025</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>Absorción Hα</t>
         </is>
       </c>
-      <c r="C7" t="n">
+      <c r="C9" t="n">
         <v>6562.948</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D9" t="n">
         <v>2.1e-05</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E9" t="n">
         <v>6.2016</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F9" t="n">
         <v>1.0973</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G9" t="n">
         <v>1.627</v>
       </c>
-      <c r="H7" t="n">
+      <c r="H9" t="n">
         <v>2.3234</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Septiembre-2025</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>6564.038</v>
+      </c>
+      <c r="D10" t="n">
+        <v>9.8e-05</v>
+      </c>
+      <c r="E10" t="n">
+        <v>29.3</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.3597</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.9419999999999999</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.3952</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Gráficos del 2025 y 2026 arreglados
</commit_message>
<xml_diff>
--- a/Datos ESPARTACO/Parámetros para análisis de Antares/resultados perfiles halpha 2025 y 2026.xlsx
+++ b/Datos ESPARTACO/Parámetros para análisis de Antares/resultados perfiles halpha 2025 y 2026.xlsx
@@ -482,22 +482,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6562.231</v>
+        <v>6562.318</v>
       </c>
       <c r="D2" t="n">
-        <v>-8.899999999999999e-05</v>
+        <v>-7.499999999999999e-05</v>
       </c>
       <c r="E2" t="n">
-        <v>-26.5631</v>
+        <v>-22.5534</v>
       </c>
       <c r="F2" t="n">
-        <v>0.3692</v>
+        <v>0.34</v>
       </c>
       <c r="G2" t="n">
-        <v>1.067</v>
+        <v>1.203</v>
       </c>
       <c r="H2" t="n">
-        <v>0.582</v>
+        <v>0.5151</v>
       </c>
     </row>
     <row r="3">
@@ -512,22 +512,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>6563.001</v>
+        <v>6562.961</v>
       </c>
       <c r="D3" t="n">
-        <v>2.9e-05</v>
+        <v>2.3e-05</v>
       </c>
       <c r="E3" t="n">
-        <v>8.641999999999999</v>
+        <v>6.7908</v>
       </c>
       <c r="F3" t="n">
-        <v>0.704</v>
+        <v>0.7534999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>1.301</v>
+        <v>1.153</v>
       </c>
       <c r="H3" t="n">
-        <v>1.2355</v>
+        <v>1.1372</v>
       </c>
     </row>
     <row r="4">
@@ -551,13 +551,13 @@
         <v>23</v>
       </c>
       <c r="F4" t="n">
-        <v>0.3432</v>
+        <v>0.4094</v>
       </c>
       <c r="G4" t="n">
-        <v>0.925</v>
+        <v>0.9419999999999999</v>
       </c>
       <c r="H4" t="n">
-        <v>0.4043</v>
+        <v>0.4855</v>
       </c>
     </row>
     <row r="5">
@@ -572,22 +572,22 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6562.453</v>
+        <v>6562.426</v>
       </c>
       <c r="D5" t="n">
-        <v>-5.5e-05</v>
+        <v>-5.9e-05</v>
       </c>
       <c r="E5" t="n">
-        <v>-16.4071</v>
+        <v>-17.612</v>
       </c>
       <c r="F5" t="n">
-        <v>0.6014</v>
+        <v>0.3264</v>
       </c>
       <c r="G5" t="n">
-        <v>1.273</v>
+        <v>1.263</v>
       </c>
       <c r="H5" t="n">
-        <v>0.9461000000000001</v>
+        <v>0.453</v>
       </c>
     </row>
     <row r="6">
@@ -602,22 +602,22 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6563.068</v>
+        <v>6563.112</v>
       </c>
       <c r="D6" t="n">
-        <v>3.9e-05</v>
+        <v>4.6e-05</v>
       </c>
       <c r="E6" t="n">
-        <v>11.7029</v>
+        <v>13.6934</v>
       </c>
       <c r="F6" t="n">
-        <v>1.033</v>
+        <v>0.8567</v>
       </c>
       <c r="G6" t="n">
-        <v>1.375</v>
+        <v>1.045</v>
       </c>
       <c r="H6" t="n">
-        <v>1.8256</v>
+        <v>1.0711</v>
       </c>
     </row>
     <row r="7">
@@ -641,13 +641,13 @@
         <v>28.7</v>
       </c>
       <c r="F7" t="n">
-        <v>0.4175</v>
+        <v>0.5532</v>
       </c>
       <c r="G7" t="n">
-        <v>0.875</v>
+        <v>0.9419999999999999</v>
       </c>
       <c r="H7" t="n">
-        <v>0.3948</v>
+        <v>0.5725</v>
       </c>
     </row>
     <row r="8">
@@ -662,22 +662,22 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>6562.469</v>
+        <v>6562.135</v>
       </c>
       <c r="D8" t="n">
-        <v>-5.2e-05</v>
+        <v>-0.000103</v>
       </c>
       <c r="E8" t="n">
-        <v>-15.6611</v>
+        <v>-30.9362</v>
       </c>
       <c r="F8" t="n">
-        <v>0.8374</v>
+        <v>0.1727</v>
       </c>
       <c r="G8" t="n">
-        <v>1.313</v>
+        <v>1.027</v>
       </c>
       <c r="H8" t="n">
-        <v>1.4598</v>
+        <v>0.2117</v>
       </c>
     </row>
     <row r="9">
@@ -692,22 +692,22 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>6562.948</v>
+        <v>6563.191</v>
       </c>
       <c r="D9" t="n">
-        <v>2.1e-05</v>
+        <v>5.8e-05</v>
       </c>
       <c r="E9" t="n">
-        <v>6.2016</v>
+        <v>17.3336</v>
       </c>
       <c r="F9" t="n">
-        <v>1.0973</v>
+        <v>0.6312</v>
       </c>
       <c r="G9" t="n">
-        <v>1.627</v>
+        <v>0.9370000000000001</v>
       </c>
       <c r="H9" t="n">
-        <v>2.3234</v>
+        <v>0.7060999999999999</v>
       </c>
     </row>
     <row r="10">
@@ -731,13 +731,13 @@
         <v>29.3</v>
       </c>
       <c r="F10" t="n">
-        <v>0.3597</v>
+        <v>0.556</v>
       </c>
       <c r="G10" t="n">
-        <v>0.9419999999999999</v>
+        <v>0.971</v>
       </c>
       <c r="H10" t="n">
-        <v>0.3952</v>
+        <v>0.6551</v>
       </c>
     </row>
   </sheetData>

</xml_diff>